<commit_message>
Add SpecificAreaCanopy into OBS datasets (via renaming or calculation)
</commit_message>
<xml_diff>
--- a/Tests/Validation/Barley/Observations/MCPD10_11Biomass.xlsx
+++ b/Tests/Validation/Barley/Observations/MCPD10_11Biomass.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHubRepos\ApsimX\Prototypes\Barley\Observations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Repos\ApsimX\Tests\Validation\Barley\Observations\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75127A4F-9BE2-4C45-A8DC-53374C49CC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15750" windowHeight="22020"/>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,9 +34,6 @@
   </si>
   <si>
     <t>Barley.Leaf.LAI</t>
-  </si>
-  <si>
-    <t>Barley.Leaf.SLA</t>
   </si>
   <si>
     <t>Barley.Grain.Wt</t>
@@ -97,11 +95,14 @@
   <si>
     <t>MCPD10_11CultRetriever</t>
   </si>
+  <si>
+    <t>Barley.Leaf.SpecificAreaCanopy</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
@@ -450,15 +451,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N73"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -469,42 +471,42 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
       </c>
       <c r="B2" s="3">
         <v>40457</v>
@@ -534,21 +536,21 @@
         <v>0</v>
       </c>
       <c r="K2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N2">
         <v>38.900000000000006</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" s="3">
         <v>40471</v>
@@ -578,21 +580,21 @@
         <v>0</v>
       </c>
       <c r="K3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N3">
         <v>111.48333333333335</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="3">
         <v>40484</v>
@@ -622,21 +624,21 @@
         <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N4">
         <v>306.5</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3">
         <v>40497</v>
@@ -666,21 +668,21 @@
         <v>0</v>
       </c>
       <c r="K5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N5">
         <v>617.01666666666665</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="3">
         <v>40504</v>
@@ -710,21 +712,21 @@
         <v>155.77083930022607</v>
       </c>
       <c r="K6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N6">
         <v>804.55201269725762</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="3">
         <v>40511</v>
@@ -754,21 +756,21 @@
         <v>255.11809142642954</v>
       </c>
       <c r="K7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N7">
         <v>1042.8664969992503</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="3">
         <v>40518</v>
@@ -798,21 +800,21 @@
         <v>503.03450064528596</v>
       </c>
       <c r="K8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N8">
         <v>1334.238004769358</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="3">
         <v>40533</v>
@@ -842,21 +844,21 @@
         <v>835.56630862246459</v>
       </c>
       <c r="K9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N9">
         <v>1572.3657090908132</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="3">
         <v>40560</v>
@@ -892,15 +894,15 @@
         <v>24470.775238150047</v>
       </c>
       <c r="M10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N10">
         <v>1533.4896096516663</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11" s="3">
         <v>40457</v>
@@ -930,21 +932,21 @@
         <v>0</v>
       </c>
       <c r="K11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N11">
         <v>23.93333333333333</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" s="3">
         <v>40471</v>
@@ -974,21 +976,21 @@
         <v>0</v>
       </c>
       <c r="K12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N12">
         <v>77.649999999999977</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="3">
         <v>40484</v>
@@ -1018,21 +1020,21 @@
         <v>0</v>
       </c>
       <c r="K13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N13">
         <v>271</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="3">
         <v>40497</v>
@@ -1062,21 +1064,21 @@
         <v>0</v>
       </c>
       <c r="K14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N14">
         <v>610</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="3">
         <v>40504</v>
@@ -1106,21 +1108,21 @@
         <v>146.68135394761768</v>
       </c>
       <c r="K15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N15">
         <v>813.95004281227557</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" s="3">
         <v>40511</v>
@@ -1150,21 +1152,21 @@
         <v>238.23663891129013</v>
       </c>
       <c r="K16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N16">
         <v>1125.1785414878811</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" s="3">
         <v>40518</v>
@@ -1194,21 +1196,21 @@
         <v>345.92631096763705</v>
       </c>
       <c r="K17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N17">
         <v>1147.3389749554242</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="3">
         <v>40533</v>
@@ -1238,21 +1240,21 @@
         <v>723.13991233664206</v>
       </c>
       <c r="K18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N18">
         <v>1440.6869239139646</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B19" s="3">
         <v>40560</v>
@@ -1288,15 +1290,15 @@
         <v>20214.368562838823</v>
       </c>
       <c r="M19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N19">
         <v>1502.145150701786</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20" s="3">
         <v>40457</v>
@@ -1326,21 +1328,21 @@
         <v>0</v>
       </c>
       <c r="K20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N20">
         <v>37.200000000000003</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21" s="3">
         <v>40471</v>
@@ -1370,21 +1372,21 @@
         <v>0</v>
       </c>
       <c r="K21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N21">
         <v>109.46666666666667</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B22" s="3">
         <v>40484</v>
@@ -1414,21 +1416,21 @@
         <v>0</v>
       </c>
       <c r="K22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N22">
         <v>357.31666666666666</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B23" s="3">
         <v>40497</v>
@@ -1458,21 +1460,21 @@
         <v>0</v>
       </c>
       <c r="K23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N23">
         <v>691.76666666666677</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B24" s="3">
         <v>40504</v>
@@ -1502,21 +1504,21 @@
         <v>157.91586524451242</v>
       </c>
       <c r="K24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N24">
         <v>836.6864136763528</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B25" s="3">
         <v>40511</v>
@@ -1546,21 +1548,21 @@
         <v>234.68496942434598</v>
       </c>
       <c r="K25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N25">
         <v>947.3046932700679</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B26" s="3">
         <v>40518</v>
@@ -1590,21 +1592,21 @@
         <v>448.65247931636333</v>
       </c>
       <c r="K26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N26">
         <v>1180.6939844828817</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B27" s="3">
         <v>40533</v>
@@ -1634,21 +1636,21 @@
         <v>809.75622725001256</v>
       </c>
       <c r="K27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N27">
         <v>1567.6966645228217</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B28" s="3">
         <v>40560</v>
@@ -1684,15 +1686,15 @@
         <v>24124.582973179509</v>
       </c>
       <c r="M28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N28">
         <v>1519.2774322839143</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B29" s="3">
         <v>40457</v>
@@ -1722,21 +1724,21 @@
         <v>0</v>
       </c>
       <c r="K29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N29">
         <v>39.950000000000003</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B30" s="3">
         <v>40471</v>
@@ -1766,21 +1768,21 @@
         <v>0</v>
       </c>
       <c r="K30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N30">
         <v>124.1</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B31" s="3">
         <v>40484</v>
@@ -1810,21 +1812,21 @@
         <v>0</v>
       </c>
       <c r="K31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N31">
         <v>300.11666666666667</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B32" s="3">
         <v>40497</v>
@@ -1854,21 +1856,21 @@
         <v>0</v>
       </c>
       <c r="K32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N32">
         <v>629.0333333333333</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B33" s="3">
         <v>40504</v>
@@ -1898,21 +1900,21 @@
         <v>126.4924845145968</v>
       </c>
       <c r="K33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N33">
         <v>775.60007719572332</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B34" s="3">
         <v>40511</v>
@@ -1942,21 +1944,21 @@
         <v>223.20003253793533</v>
       </c>
       <c r="K34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N34">
         <v>1035.0231497606455</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B35" s="3">
         <v>40518</v>
@@ -1986,21 +1988,21 @@
         <v>393.44289749541616</v>
       </c>
       <c r="K35" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L35" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M35" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N35">
         <v>1238.638921243255</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B36" s="3">
         <v>40533</v>
@@ -2030,21 +2032,21 @@
         <v>834.0196232374243</v>
       </c>
       <c r="K36" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L36" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M36" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N36">
         <v>1687.256555245101</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B37" s="3">
         <v>40560</v>
@@ -2080,15 +2082,15 @@
         <v>22042.734077466084</v>
       </c>
       <c r="M37" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N37">
         <v>1534.0305323703301</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B38" s="3">
         <v>40457</v>
@@ -2118,21 +2120,21 @@
         <v>0</v>
       </c>
       <c r="K38" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L38" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M38" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N38">
         <v>53.599999999999994</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B39" s="3">
         <v>40471</v>
@@ -2162,21 +2164,21 @@
         <v>0</v>
       </c>
       <c r="K39" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L39" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M39" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N39">
         <v>187.31666666666666</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B40" s="3">
         <v>40484</v>
@@ -2206,21 +2208,21 @@
         <v>0</v>
       </c>
       <c r="K40" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L40" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M40" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N40">
         <v>410.7833333333333</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B41" s="3">
         <v>40497</v>
@@ -2250,21 +2252,21 @@
         <v>0</v>
       </c>
       <c r="K41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N41">
         <v>692.05</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B42" s="3">
         <v>40504</v>
@@ -2294,21 +2296,21 @@
         <v>180.27258789633305</v>
       </c>
       <c r="K42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N42">
         <v>963.37433823680908</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B43" s="3">
         <v>40511</v>
@@ -2338,21 +2340,21 @@
         <v>252.45701404207267</v>
       </c>
       <c r="K43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N43">
         <v>1070.0182099427257</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B44" s="3">
         <v>40518</v>
@@ -2382,21 +2384,21 @@
         <v>416.8596315513376</v>
       </c>
       <c r="K44" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L44" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M44" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N44">
         <v>1239.7047394303959</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B45" s="3">
         <v>40533</v>
@@ -2426,21 +2428,21 @@
         <v>836.75347762971739</v>
       </c>
       <c r="K45" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L45" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M45" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N45">
         <v>1691.5718212291288</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B46" s="3">
         <v>40560</v>
@@ -2476,15 +2478,15 @@
         <v>20386.965840912151</v>
       </c>
       <c r="M46" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N46">
         <v>1621.0631303774067</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B47" s="3">
         <v>40457</v>
@@ -2514,21 +2516,21 @@
         <v>0</v>
       </c>
       <c r="K47" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L47" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M47" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N47">
         <v>29.966666666666669</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B48" s="3">
         <v>40471</v>
@@ -2558,21 +2560,21 @@
         <v>0</v>
       </c>
       <c r="K48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N48">
         <v>95.616666666666674</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B49" s="3">
         <v>40484</v>
@@ -2602,21 +2604,21 @@
         <v>0</v>
       </c>
       <c r="K49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N49">
         <v>282.25</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B50" s="3">
         <v>40497</v>
@@ -2646,21 +2648,21 @@
         <v>0</v>
       </c>
       <c r="K50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N50">
         <v>571.81666666666661</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B51" s="3">
         <v>40504</v>
@@ -2690,21 +2692,21 @@
         <v>160.0438737324682</v>
       </c>
       <c r="K51" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L51" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M51" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N51">
         <v>858.79044752535879</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B52" s="3">
         <v>40511</v>
@@ -2734,21 +2736,21 @@
         <v>239.50127202675236</v>
       </c>
       <c r="K52" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L52" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M52" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N52">
         <v>1061.2862785222219</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B53" s="3">
         <v>40518</v>
@@ -2778,21 +2780,21 @@
         <v>427.33222221207313</v>
       </c>
       <c r="K53" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L53" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M53" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N53">
         <v>1247.946345190815</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B54" s="3">
         <v>40533</v>
@@ -2822,21 +2824,21 @@
         <v>772.68592201908564</v>
       </c>
       <c r="K54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N54">
         <v>1525.6879637555598</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B55" s="3">
         <v>40560</v>
@@ -2872,15 +2874,15 @@
         <v>23374.586083643193</v>
       </c>
       <c r="M55" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N55">
         <v>1539.9921609557525</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B56" s="3">
         <v>40457</v>
@@ -2910,21 +2912,21 @@
         <v>0</v>
       </c>
       <c r="K56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N56">
         <v>28.450000000000003</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B57" s="3">
         <v>40471</v>
@@ -2954,21 +2956,21 @@
         <v>0</v>
       </c>
       <c r="K57" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L57" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M57" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N57">
         <v>104.21666666666667</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B58" s="3">
         <v>40484</v>
@@ -2998,21 +3000,21 @@
         <v>0</v>
       </c>
       <c r="K58" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L58" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M58" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N58">
         <v>289.2166666666667</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B59" s="3">
         <v>40497</v>
@@ -3042,21 +3044,21 @@
         <v>0</v>
       </c>
       <c r="K59" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L59" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M59" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N59">
         <v>561.7166666666667</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B60" s="3">
         <v>40504</v>
@@ -3086,21 +3088,21 @@
         <v>188.46887970747193</v>
       </c>
       <c r="K60" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L60" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M60" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N60">
         <v>816.08203575754578</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B61" s="3">
         <v>40511</v>
@@ -3130,21 +3132,21 @@
         <v>274.31247217724973</v>
       </c>
       <c r="K61" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L61" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M61" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N61">
         <v>1174.7971559857901</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B62" s="3">
         <v>40518</v>
@@ -3174,21 +3176,21 @@
         <v>406.59963077389364</v>
       </c>
       <c r="K62" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L62" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M62" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N62">
         <v>1258.5509903386696</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B63" s="3">
         <v>40533</v>
@@ -3218,21 +3220,21 @@
         <v>871.19261089437225</v>
       </c>
       <c r="K63" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L63" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M63" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N63">
         <v>1645.5554627206709</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B64" s="3">
         <v>40560</v>
@@ -3268,15 +3270,15 @@
         <v>24828.142117091378</v>
       </c>
       <c r="M64" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N64">
         <v>1671.6329663639344</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B65" s="3">
         <v>40457</v>
@@ -3306,21 +3308,21 @@
         <v>0</v>
       </c>
       <c r="K65" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L65" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M65" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N65">
         <v>42.333333333333336</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B66" s="3">
         <v>40471</v>
@@ -3350,21 +3352,21 @@
         <v>0</v>
       </c>
       <c r="K66" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L66" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M66" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N66">
         <v>101.80000000000001</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B67" s="3">
         <v>40484</v>
@@ -3394,21 +3396,21 @@
         <v>0</v>
       </c>
       <c r="K67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N67">
         <v>193.43333333333334</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B68" s="3">
         <v>40497</v>
@@ -3438,21 +3440,21 @@
         <v>0</v>
       </c>
       <c r="K68" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L68" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M68" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N68">
         <v>458.2</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B69" s="3">
         <v>40504</v>
@@ -3482,21 +3484,21 @@
         <v>76.92629004941108</v>
       </c>
       <c r="K69" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L69" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M69" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N69">
         <v>753.95</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B70" s="3">
         <v>40511</v>
@@ -3526,21 +3528,21 @@
         <v>191.32172357853594</v>
       </c>
       <c r="K70" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L70" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M70" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N70">
         <v>898.08334421697668</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B71" s="3">
         <v>40518</v>
@@ -3570,21 +3572,21 @@
         <v>290.88039367083417</v>
       </c>
       <c r="K71" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L71" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M71" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N71">
         <v>1151.0125108451618</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B72" s="3">
         <v>40533</v>
@@ -3614,21 +3616,21 @@
         <v>593.12785213636607</v>
       </c>
       <c r="K72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N72">
         <v>1339.9372500936429</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B73" s="3">
         <v>40560</v>
@@ -3664,7 +3666,7 @@
         <v>18583.944640113357</v>
       </c>
       <c r="M73" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N73">
         <v>1525.0212431250479</v>

</xml_diff>